<commit_message>
chore: refresh complete MF holdings
</commit_message>
<xml_diff>
--- a/data/Networth_Raw_Data.xlsx
+++ b/data/Networth_Raw_Data.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -495,7 +495,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>SAMPLE-100</t>
+          <t>SAMPLE-200</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -543,7 +543,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SAMPLE-101</t>
+          <t>SAMPLE-201</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -591,7 +591,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SAMPLE-102</t>
+          <t>SAMPLE-202</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -601,12 +601,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2024-01-15</t>
+          <t>2019-09-17</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2027-01-15</t>
+          <t>2027-01-01</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -615,46 +615,46 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>100000</v>
+        <v>72029</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>100000</v>
+        <v>72029</v>
       </c>
       <c r="I4" t="n">
-        <v>119000</v>
+        <v>77097</v>
       </c>
       <c r="J4" t="n">
-        <v>6.5</v>
+        <v>6.25</v>
       </c>
       <c r="K4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L4" t="n">
-        <v>36</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SAMPLE-103</t>
+          <t>SAMPLE-203</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Member B</t>
+          <t>Member A</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2023-06-01</t>
+          <t>2023-10-16</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2027-01-25</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -663,46 +663,46 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>200000</v>
+        <v>54960</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>200000</v>
+        <v>54960</v>
       </c>
       <c r="I5" t="n">
-        <v>240000</v>
+        <v>58817</v>
       </c>
       <c r="J5" t="n">
-        <v>6.4</v>
+        <v>6.25</v>
       </c>
       <c r="K5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L5" t="n">
-        <v>36</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SAMPLE-104</t>
+          <t>SAMPLE-204</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Member B</t>
+          <t>Member D</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2022-03-10</t>
+          <t>2025-10-07</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2027-03-10</t>
+          <t>2026-11-07</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -711,46 +711,46 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>150000</v>
+        <v>200000</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>150000</v>
+        <v>200000</v>
       </c>
       <c r="I6" t="n">
-        <v>195000</v>
+        <v>215072</v>
       </c>
       <c r="J6" t="n">
-        <v>6.5</v>
+        <v>6.75</v>
       </c>
       <c r="K6" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="L6" t="n">
-        <v>60</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SAMPLE-105</t>
+          <t>SAMPLE-205</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Member C</t>
+          <t>Member D</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2021-08-20</t>
+          <t>2025-04-24</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2027-04-24</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -759,31 +759,31 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>75000</v>
+        <v>300000</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>75000</v>
+        <v>300000</v>
       </c>
       <c r="I7" t="n">
-        <v>98000</v>
+        <v>347384</v>
       </c>
       <c r="J7" t="n">
-        <v>6.2</v>
+        <v>7.4</v>
       </c>
       <c r="K7" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L7" t="n">
-        <v>60</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SAMPLE-106</t>
+          <t>SAMPLE-206</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -793,12 +793,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2020-11-05</t>
+          <t>2023-06-15</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2025-11-05</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -807,25 +807,793 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>50000</v>
+        <v>77621</v>
       </c>
       <c r="G8" t="n">
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>50000</v>
+        <v>77621</v>
       </c>
       <c r="I8" t="n">
-        <v>65000</v>
+        <v>83532</v>
       </c>
       <c r="J8" t="n">
-        <v>6</v>
+        <v>6.75</v>
       </c>
       <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>SAMPLE-207</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Member B</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2028-01-07</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>7467.76</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>7467.76</v>
+      </c>
+      <c r="I9" t="n">
+        <v>8199.139999999999</v>
+      </c>
+      <c r="J9" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="K9" t="n">
+        <v>1</v>
+      </c>
+      <c r="L9" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>SAMPLE-208</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Member B</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2025-10-14</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>7324.09</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>7324.09</v>
+      </c>
+      <c r="I10" t="n">
+        <v>7695.38</v>
+      </c>
+      <c r="J10" t="n">
         <v>5</v>
       </c>
-      <c r="L8" t="n">
-        <v>60</v>
+      <c r="K10" t="n">
+        <v>1</v>
+      </c>
+      <c r="L10" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>SAMPLE-209</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Member B</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2029-08-26</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>7695.16</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>7695.16</v>
+      </c>
+      <c r="I11" t="n">
+        <v>9281.24</v>
+      </c>
+      <c r="J11" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="K11" t="n">
+        <v>3</v>
+      </c>
+      <c r="L11" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>SAMPLE-210</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Member B</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2025-04-08</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2027-03-08</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>9530.309999999999</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="n">
+        <v>9530.309999999999</v>
+      </c>
+      <c r="I12" t="n">
+        <v>10589.52</v>
+      </c>
+      <c r="J12" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="K12" t="n">
+        <v>1</v>
+      </c>
+      <c r="L12" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>SAMPLE-211</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Member B</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2025-01-15</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2026-12-15</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>6732.37</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="n">
+        <v>6732.37</v>
+      </c>
+      <c r="I13" t="n">
+        <v>7480.61</v>
+      </c>
+      <c r="J13" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="K13" t="n">
+        <v>1</v>
+      </c>
+      <c r="L13" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>SAMPLE-212</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Member B</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>2029-09-01</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>11600.12</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="n">
+        <v>11600.12</v>
+      </c>
+      <c r="I14" t="n">
+        <v>12325.1275</v>
+      </c>
+      <c r="J14" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="K14" t="n">
+        <v>3</v>
+      </c>
+      <c r="L14" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>SAMPLE-213</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Member B</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>2024-07-05</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>2028-05-05</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>7537.41</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="n">
+        <v>7537.41</v>
+      </c>
+      <c r="I15" t="n">
+        <v>8203.25</v>
+      </c>
+      <c r="J15" t="n">
+        <v>5.65</v>
+      </c>
+      <c r="K15" t="n">
+        <v>1</v>
+      </c>
+      <c r="L15" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>SAMPLE-214</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Member B</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>2024-01-09</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>2027-01-09</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>7725.96</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" t="n">
+        <v>7725.96</v>
+      </c>
+      <c r="I16" t="n">
+        <v>8094.12</v>
+      </c>
+      <c r="J16" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="K16" t="n">
+        <v>1</v>
+      </c>
+      <c r="L16" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>SAMPLE-215</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Member B</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>2027-04-22</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>7828.35</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="n">
+        <v>7929.77</v>
+      </c>
+      <c r="I17" t="n">
+        <v>8177.58</v>
+      </c>
+      <c r="J17" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="K17" t="n">
+        <v>1</v>
+      </c>
+      <c r="L17" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>SAMPLE-216</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Member B</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>2025-02-10</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>2027-04-21</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>422022</v>
+      </c>
+      <c r="G18" t="n">
+        <v>400000</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" t="n">
+        <v>451714</v>
+      </c>
+      <c r="J18" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>SAMPLE-217</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Member B</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>2021-10-26</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>2027-10-26</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>2342229</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" t="n">
+        <v>2342229</v>
+      </c>
+      <c r="I19" t="n">
+        <v>2863124</v>
+      </c>
+      <c r="J19" t="n">
+        <v>6.75</v>
+      </c>
+      <c r="K19" t="n">
+        <v>3</v>
+      </c>
+      <c r="L19" t="n">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>SAMPLE-218</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Member B</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>2029-07-08</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>7690.81</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" t="n">
+        <v>7690.81</v>
+      </c>
+      <c r="I20" t="n">
+        <v>9005.41</v>
+      </c>
+      <c r="J20" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="K20" t="n">
+        <v>3</v>
+      </c>
+      <c r="L20" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>SAMPLE-219</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Member B</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>2029-08-01</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>7000</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" t="n">
+        <v>7000</v>
+      </c>
+      <c r="I21" t="n">
+        <v>8442.809999999999</v>
+      </c>
+      <c r="J21" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="K21" t="n">
+        <v>3</v>
+      </c>
+      <c r="L21" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>SAMPLE-220</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Member B</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>2029-08-01</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>7000</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" t="n">
+        <v>7000</v>
+      </c>
+      <c r="I22" t="n">
+        <v>8442.809999999999</v>
+      </c>
+      <c r="J22" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="K22" t="n">
+        <v>3</v>
+      </c>
+      <c r="L22" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>SAMPLE-221</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Member B</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>2029-08-01</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>7000</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" t="n">
+        <v>7000</v>
+      </c>
+      <c r="I23" t="n">
+        <v>8442.809999999999</v>
+      </c>
+      <c r="J23" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="K23" t="n">
+        <v>3</v>
+      </c>
+      <c r="L23" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>SAMPLE-222</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Member B</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>2029-08-01</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>7000</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" t="n">
+        <v>7000</v>
+      </c>
+      <c r="I24" t="n">
+        <v>8442.809999999999</v>
+      </c>
+      <c r="J24" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="K24" t="n">
+        <v>3</v>
+      </c>
+      <c r="L24" t="n">
+        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>